<commit_message>
Anchor gap analysis in mainframe source with Python satisfaction evidence
Require source-led comparisons with original mainframe logic on the left and actual Python code, satisfaction explanation, evidence and remaining gaps on the right. Preserve unmatched and non-executable source dispositions. Add the aligned Gap Analysis workbook view and update specialist instructions and the specification.

Kit checks and workbook preservation/visual checks pass. No mainframe conversion or execution is claimed.
</commit_message>
<xml_diff>
--- a/examples/PTS_Modernization_Review_Template.xlsx
+++ b/examples/PTS_Modernization_Review_Template.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SME Review" sheetId="1" r:id="Ra5117f20562a4713"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Process Intake" sheetId="2" r:id="R3c2e091377cc475a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Converted Inventory" sheetId="3" r:id="Rf267421b7960407f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Evidence" sheetId="4" r:id="R51b91305490f4350"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow" sheetId="5" r:id="Refca00a49af84908"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Illustrative Review" sheetId="6" r:id="R53f4c24b10494462"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Catalog" sheetId="7" r:id="R7f13e33a99ac4d4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Map" sheetId="8" r:id="Rdb972b5afc354ee9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SME Review" sheetId="1" r:id="R2eb1be4d55804bde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Process Intake" sheetId="2" r:id="R30c7464998954f0b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Converted Inventory" sheetId="3" r:id="Re84e38142441422e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Evidence" sheetId="4" r:id="Re73fddde36664568"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow" sheetId="5" r:id="Ra78013c3b06c440d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Illustrative Review" sheetId="6" r:id="R94b494bf73b7446a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Catalog" sheetId="7" r:id="Re550f38ff7ee4217"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Map" sheetId="8" r:id="R55ca45ad68684924"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Analysis" sheetId="9" r:id="R1416bde0c4004bb8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +26,7 @@
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -52,8 +53,26 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF253B53"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FF253B53"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FF627287"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -80,8 +99,33 @@
         <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE8EEF5"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF1F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF253B53"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF1F5F9"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="5">
+  <x:borders count="7">
     <x:border>
       <x:left/>
       <x:right/>
@@ -127,11 +171,31 @@
       <x:bottom/>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left style="medium">
+        <x:color rgb="FF8795A6"/>
+      </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="medium">
+        <x:color rgb="FF8795A6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFFFFFFF"/>
+      </x:right>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="46">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -209,18 +273,92 @@
     <x:xf numFmtId="202" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
+  <x:dxfs count="5">
     <x:dxf>
       <x:font>
         <x:color rgb="FF9C2F2F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE6E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF9C2F2F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE6E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -349,6 +487,21 @@
     <x:tableColumn id="2" name="Skills"/>
     <x:tableColumn id="3" name="Required input"/>
     <x:tableColumn id="4" name="Expected output"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="MainframePythonGap" displayName="MainframePythonGap" ref="A6:F26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A6:F26"/>
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="Mainframe unit / source reference"/>
+    <x:tableColumn id="2" name="Mainframe behavior / source code"/>
+    <x:tableColumn id="3" name="Python code / source reference"/>
+    <x:tableColumn id="4" name="How Python satisfies the behavior"/>
+    <x:tableColumn id="5" name="Coverage status"/>
+    <x:tableColumn id="6" name="Evidence, gap and next action"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -791,7 +944,7 @@
     </x:row>
     <x:row r="4" ht="27" customHeight="1">
       <x:c r="A4" s="7" t="str">
-        <x:v>Source and target evidence are populated during analysis. No repository source has been imported into this template.</x:v>
+        <x:v>See Gap Analysis for mainframe logic on the left and the Python code, explanation and evidence on the right.</x:v>
       </x:c>
       <x:c r="B4" s="2"/>
       <x:c r="C4" s="2"/>
@@ -1379,7 +1532,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R393d9511d17a4cee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3ac707b61dc4106"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2134,8 +2287,8 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8358db9f8b640dd"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12e51dbc65c24677"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55b8a7ab184c4a6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1190d74440a2455e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2708,7 +2861,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5556c4e01e1438c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d9e89f734f8419e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3511,7 +3664,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3481838cf10749e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa7f9e3765014dcd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3545,7 +3698,7 @@
     </x:row>
     <x:row r="3" ht="27" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>Operating contract, version 4.0. Claude Code lead + eight specialist roles; three core skills; no custom orchestration engine.</x:v>
+        <x:v>Operating contract, version 4.1. Claude Code lead + eight specialist roles; three core skills; mainframe-based gap analysis.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -3601,10 +3754,10 @@
         <x:v>Gap analysis + design</x:v>
       </x:c>
       <x:c r="C8" s="17" t="str">
-        <x:v>Classify business, technical, mixed and unknown units per program. Resolve process → jobs → steps → programs and dependencies. Account for every source span.</x:v>
+        <x:v>Derive every requirement from mainframe source first. Classify each unit and account for every source span. Gap Analysis shows mainframe logic on the left and Python implementation, explanation, evidence and gaps on the right.</x:v>
       </x:c>
       <x:c r="D8" s="17" t="str">
-        <x:v>Dependency graph + source coverage ledger</x:v>
+        <x:v>Source-based requirements + initial Gap Analysis with missing target rows retained</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="95" customHeight="1">
@@ -3643,10 +3796,10 @@
         <x:v>Backend + frontend</x:v>
       </x:c>
       <x:c r="C11" s="16" t="str">
-        <x:v>Use minimal Python, SQL and existing Sparkflows flows. Separate business rules and database adapters. Build only needed record/SME views. Preserve source-to-code and source-to-flow mappings.</x:v>
+        <x:v>Use minimal Python, SQL and existing Sparkflows flows. Update each mainframe requirement with exact Python code, location and explanation of how it satisfies the behavior. Link delegated SQL/ETL and refresh gap status.</x:v>
       </x:c>
       <x:c r="D11" s="16" t="str">
-        <x:v>Versioned code/flow + source mapping + benchmark</x:v>
+        <x:v>Versioned implementation + updated source-to-Python comparison</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="95" customHeight="1">
@@ -4372,11 +4525,11 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="5">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra556d88cd1ce4c67"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c571c9bab064dd3"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fc213e927e64495"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffc2bcdb8fdc47a2"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb45a67bb5bbc4b46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b860873699b4f56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea9883b517f44aa9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0750ed0dab6b4742"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33ff0eb6afab430d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2d37593cb4f4711"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5132,7 +5285,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75fcfc898a044f18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5299e3b007914a9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5618,7 +5771,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91bea64a64a94dc2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf76df2a81ed4a8c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5801,10 +5954,10 @@
         <x:v>modernize-process; consult-modernization</x:v>
       </x:c>
       <x:c r="C15" s="16" t="str">
-        <x:v>Complete approved source inventory, JCL, copybooks, dependencies and knowledge</x:v>
+        <x:v>Mainframe source inventory, JCL, copybooks and dependencies first; then current Python/SQL/ETL and actual test evidence</x:v>
       </x:c>
       <x:c r="D15" s="16" t="str">
-        <x:v>All-program classification, source ledger, dependency graph and focused SME questions</x:v>
+        <x:v>Mainframe on the left, Python code and satisfaction evidence on the right; explicit missing/partial behavior and next actions</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="27" customHeight="1">
@@ -5870,7 +6023,427 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re316a4128b30470e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66a0109396b74eaf"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF253B53"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="35.560001373291016" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="35.560001373291016" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="35.560001373291016" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22.219999313354492" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="37.779998779296875" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="27" customHeight="1">
+      <x:c r="A1" s="2"/>
+      <x:c r="B1" s="2"/>
+      <x:c r="C1" s="2"/>
+      <x:c r="D1" s="2"/>
+      <x:c r="E1" s="2"/>
+      <x:c r="F1" s="2"/>
+    </x:row>
+    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="A2" s="4" t="str">
+        <x:v>Mainframe to Python gap analysis</x:v>
+      </x:c>
+      <x:c r="B2" s="5"/>
+      <x:c r="C2" s="5"/>
+      <x:c r="D2" s="5"/>
+      <x:c r="E2" s="5"/>
+      <x:c r="F2" s="5"/>
+    </x:row>
+    <x:row r="3" ht="27" customHeight="1">
+      <x:c r="A3" s="7" t="str">
+        <x:v>Each row starts from the mainframe. Engineering fills the Python mapping and evidence. Missing implementations remain visible.</x:v>
+      </x:c>
+      <x:c r="B3" s="7"/>
+      <x:c r="C3" s="7"/>
+      <x:c r="D3" s="7"/>
+      <x:c r="E3" s="7"/>
+      <x:c r="F3" s="7"/>
+    </x:row>
+    <x:row r="4" ht="27" customHeight="1">
+      <x:c r="A4" s="7" t="str">
+        <x:v>Generated from source-map.json. Unit evidence and observed mainframe parity stay separate; changes require an SME decision reference.</x:v>
+      </x:c>
+      <x:c r="B4" s="7"/>
+      <x:c r="C4" s="7"/>
+      <x:c r="D4" s="7"/>
+      <x:c r="E4" s="7"/>
+      <x:c r="F4" s="7"/>
+    </x:row>
+    <x:row r="5" ht="27" customHeight="1">
+      <x:c r="A5" s="29" t="str">
+        <x:v>MAINFRAME BASELINE</x:v>
+      </x:c>
+      <x:c r="B5" s="29"/>
+      <x:c r="C5" s="40" t="str">
+        <x:v>PYTHON IMPLEMENTATION AND EVIDENCE</x:v>
+      </x:c>
+      <x:c r="D5" s="30"/>
+      <x:c r="E5" s="30"/>
+      <x:c r="F5" s="30"/>
+    </x:row>
+    <x:row r="6" ht="48" customHeight="1">
+      <x:c r="A6" s="35" t="str">
+        <x:v>Mainframe unit / source reference</x:v>
+      </x:c>
+      <x:c r="B6" s="36" t="str">
+        <x:v>Mainframe behavior / source code</x:v>
+      </x:c>
+      <x:c r="C6" s="41" t="str">
+        <x:v>Python code / source reference</x:v>
+      </x:c>
+      <x:c r="D6" s="36" t="str">
+        <x:v>How Python satisfies the behavior</x:v>
+      </x:c>
+      <x:c r="E6" s="36" t="str">
+        <x:v>Coverage status</x:v>
+      </x:c>
+      <x:c r="F6" s="37" t="str">
+        <x:v>Evidence, gap and next action</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="96" customHeight="1">
+      <x:c r="A7" s="38"/>
+      <x:c r="B7" s="38"/>
+      <x:c r="C7" s="42"/>
+      <x:c r="D7" s="38"/>
+      <x:c r="E7" s="38"/>
+      <x:c r="F7" s="38"/>
+    </x:row>
+    <x:row r="8" ht="96" customHeight="1">
+      <x:c r="A8" s="39"/>
+      <x:c r="B8" s="39"/>
+      <x:c r="C8" s="43"/>
+      <x:c r="D8" s="39"/>
+      <x:c r="E8" s="39"/>
+      <x:c r="F8" s="39"/>
+    </x:row>
+    <x:row r="9" ht="96" customHeight="1">
+      <x:c r="A9" s="38"/>
+      <x:c r="B9" s="38"/>
+      <x:c r="C9" s="42"/>
+      <x:c r="D9" s="38"/>
+      <x:c r="E9" s="38"/>
+      <x:c r="F9" s="38"/>
+    </x:row>
+    <x:row r="10" ht="96" customHeight="1">
+      <x:c r="A10" s="39"/>
+      <x:c r="B10" s="39"/>
+      <x:c r="C10" s="43"/>
+      <x:c r="D10" s="39"/>
+      <x:c r="E10" s="39"/>
+      <x:c r="F10" s="39"/>
+    </x:row>
+    <x:row r="11" ht="96" customHeight="1">
+      <x:c r="A11" s="38"/>
+      <x:c r="B11" s="38"/>
+      <x:c r="C11" s="42"/>
+      <x:c r="D11" s="38"/>
+      <x:c r="E11" s="38"/>
+      <x:c r="F11" s="38"/>
+    </x:row>
+    <x:row r="12" ht="96" customHeight="1">
+      <x:c r="A12" s="39"/>
+      <x:c r="B12" s="39"/>
+      <x:c r="C12" s="43"/>
+      <x:c r="D12" s="39"/>
+      <x:c r="E12" s="39"/>
+      <x:c r="F12" s="39"/>
+    </x:row>
+    <x:row r="13" ht="96" customHeight="1">
+      <x:c r="A13" s="38"/>
+      <x:c r="B13" s="38"/>
+      <x:c r="C13" s="42"/>
+      <x:c r="D13" s="38"/>
+      <x:c r="E13" s="38"/>
+      <x:c r="F13" s="38"/>
+    </x:row>
+    <x:row r="14" ht="96" customHeight="1">
+      <x:c r="A14" s="39"/>
+      <x:c r="B14" s="39"/>
+      <x:c r="C14" s="43"/>
+      <x:c r="D14" s="39"/>
+      <x:c r="E14" s="39"/>
+      <x:c r="F14" s="39"/>
+    </x:row>
+    <x:row r="15" ht="96" customHeight="1">
+      <x:c r="A15" s="38"/>
+      <x:c r="B15" s="38"/>
+      <x:c r="C15" s="42"/>
+      <x:c r="D15" s="38"/>
+      <x:c r="E15" s="38"/>
+      <x:c r="F15" s="38"/>
+    </x:row>
+    <x:row r="16" ht="96" customHeight="1">
+      <x:c r="A16" s="39"/>
+      <x:c r="B16" s="39"/>
+      <x:c r="C16" s="43"/>
+      <x:c r="D16" s="39"/>
+      <x:c r="E16" s="39"/>
+      <x:c r="F16" s="39"/>
+    </x:row>
+    <x:row r="17" ht="96" customHeight="1">
+      <x:c r="A17" s="38"/>
+      <x:c r="B17" s="38"/>
+      <x:c r="C17" s="42"/>
+      <x:c r="D17" s="38"/>
+      <x:c r="E17" s="38"/>
+      <x:c r="F17" s="38"/>
+    </x:row>
+    <x:row r="18" ht="96" customHeight="1">
+      <x:c r="A18" s="39"/>
+      <x:c r="B18" s="39"/>
+      <x:c r="C18" s="43"/>
+      <x:c r="D18" s="39"/>
+      <x:c r="E18" s="39"/>
+      <x:c r="F18" s="39"/>
+    </x:row>
+    <x:row r="19" ht="96" customHeight="1">
+      <x:c r="A19" s="38"/>
+      <x:c r="B19" s="38"/>
+      <x:c r="C19" s="42"/>
+      <x:c r="D19" s="38"/>
+      <x:c r="E19" s="38"/>
+      <x:c r="F19" s="38"/>
+    </x:row>
+    <x:row r="20" ht="96" customHeight="1">
+      <x:c r="A20" s="39"/>
+      <x:c r="B20" s="39"/>
+      <x:c r="C20" s="43"/>
+      <x:c r="D20" s="39"/>
+      <x:c r="E20" s="39"/>
+      <x:c r="F20" s="39"/>
+    </x:row>
+    <x:row r="21" ht="96" customHeight="1">
+      <x:c r="A21" s="38"/>
+      <x:c r="B21" s="38"/>
+      <x:c r="C21" s="42"/>
+      <x:c r="D21" s="38"/>
+      <x:c r="E21" s="38"/>
+      <x:c r="F21" s="38"/>
+    </x:row>
+    <x:row r="22" ht="96" customHeight="1">
+      <x:c r="A22" s="39"/>
+      <x:c r="B22" s="39"/>
+      <x:c r="C22" s="43"/>
+      <x:c r="D22" s="39"/>
+      <x:c r="E22" s="39"/>
+      <x:c r="F22" s="39"/>
+    </x:row>
+    <x:row r="23" ht="96" customHeight="1">
+      <x:c r="A23" s="38"/>
+      <x:c r="B23" s="38"/>
+      <x:c r="C23" s="42"/>
+      <x:c r="D23" s="38"/>
+      <x:c r="E23" s="38"/>
+      <x:c r="F23" s="38"/>
+    </x:row>
+    <x:row r="24" ht="96" customHeight="1">
+      <x:c r="A24" s="39"/>
+      <x:c r="B24" s="39"/>
+      <x:c r="C24" s="43"/>
+      <x:c r="D24" s="39"/>
+      <x:c r="E24" s="39"/>
+      <x:c r="F24" s="39"/>
+    </x:row>
+    <x:row r="25" ht="96" customHeight="1">
+      <x:c r="A25" s="38"/>
+      <x:c r="B25" s="38"/>
+      <x:c r="C25" s="42"/>
+      <x:c r="D25" s="38"/>
+      <x:c r="E25" s="38"/>
+      <x:c r="F25" s="38"/>
+    </x:row>
+    <x:row r="26" ht="96" customHeight="1">
+      <x:c r="A26" s="39"/>
+      <x:c r="B26" s="39"/>
+      <x:c r="C26" s="43"/>
+      <x:c r="D26" s="39"/>
+      <x:c r="E26" s="39"/>
+      <x:c r="F26" s="39"/>
+    </x:row>
+    <x:row r="27" ht="27" customHeight="1">
+      <x:c r="A27" s="2"/>
+      <x:c r="B27" s="2"/>
+      <x:c r="C27" s="2"/>
+      <x:c r="D27" s="2"/>
+      <x:c r="E27" s="2"/>
+      <x:c r="F27" s="2"/>
+    </x:row>
+    <x:row r="28" ht="27" customHeight="1">
+      <x:c r="A28" s="44" t="str">
+        <x:v>Required row content</x:v>
+      </x:c>
+      <x:c r="B28" s="2"/>
+      <x:c r="C28" s="2"/>
+      <x:c r="D28" s="2"/>
+      <x:c r="E28" s="2"/>
+      <x:c r="F28" s="2"/>
+    </x:row>
+    <x:row r="29" ht="128" customHeight="1">
+      <x:c r="A29" s="15" t="str">
+        <x:v>Program + stable unit ID, class, dataset/member, immutable source hash/version and original lines. Link additional spans.</x:v>
+      </x:c>
+      <x:c r="B29" s="15" t="str">
+        <x:v>Exact approved source excerpt plus condition, expected outcomes and side effects. Derive this before inspecting Python.</x:v>
+      </x:c>
+      <x:c r="C29" s="15" t="str">
+        <x:v>Current Python path, hash/version, function and lines, with exact relevant code. Use Missing when absent; label proposed code.</x:v>
+      </x:c>
+      <x:c r="D29" s="15" t="str">
+        <x:v>Explain condition, values, state and effects. Link the actual SQL/ETL artifact when behavior is delegated. Do not add Python wrappers for this view.</x:v>
+      </x:c>
+      <x:c r="E29" s="15" t="str">
+        <x:v>Status follows evidence. Non-executable source needs a reason. Approved change/removal needs a decision. Neither means equivalent behavior.</x:v>
+      </x:c>
+      <x:c r="F29" s="15" t="str">
+        <x:v>Case/run IDs and results, observed legacy comparison or unavailable, decision IDs, specific remaining gap, next action and owner.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="27" customHeight="1">
+      <x:c r="A30" s="2"/>
+      <x:c r="B30" s="2"/>
+      <x:c r="C30" s="2"/>
+      <x:c r="D30" s="2"/>
+      <x:c r="E30" s="2"/>
+      <x:c r="F30" s="2"/>
+    </x:row>
+    <x:row r="31" ht="27" customHeight="1">
+      <x:c r="A31" s="45" t="str">
+        <x:v>Fictional format example — no PTS source or execution evidence</x:v>
+      </x:c>
+      <x:c r="B31" s="2"/>
+      <x:c r="C31" s="2"/>
+      <x:c r="D31" s="2"/>
+      <x:c r="E31" s="2"/>
+      <x:c r="F31" s="2"/>
+    </x:row>
+    <x:row r="32" ht="48" customHeight="1">
+      <x:c r="A32" s="35" t="str">
+        <x:v>Mainframe unit / source reference</x:v>
+      </x:c>
+      <x:c r="B32" s="36" t="str">
+        <x:v>Mainframe behavior / source code</x:v>
+      </x:c>
+      <x:c r="C32" s="36" t="str">
+        <x:v>Python code / source reference</x:v>
+      </x:c>
+      <x:c r="D32" s="36" t="str">
+        <x:v>How Python satisfies the behavior</x:v>
+      </x:c>
+      <x:c r="E32" s="36" t="str">
+        <x:v>Coverage status</x:v>
+      </x:c>
+      <x:c r="F32" s="37" t="str">
+        <x:v>Evidence, gap and next action</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="178" customHeight="1">
+      <x:c r="A33" s="39" t="str">
+        <x:v>FICTIONAL A1
+EX-A1-U001 · Business
+demo/A1.cbl:100–102
+Source version/hash: example only</x:v>
+      </x:c>
+      <x:c r="B33" s="39" t="str">
+        <x:v>Set the review flag to Y when the amount is negative; otherwise preserve its incoming value.
+IF AMOUNT &lt; ZERO
+    MOVE "Y" TO REVIEW-FLAG
+END-IF</x:v>
+      </x:c>
+      <x:c r="C33" s="39" t="str">
+        <x:v>FICTIONAL target/a1.py:1–4
+Version/hash: example only
+def flag_negative(amount, flag):
+    if amount &lt; 0:
+        flag = "Y"
+    return flag</x:v>
+      </x:c>
+      <x:c r="D33" s="39" t="str">
+        <x:v>The &lt; 0 condition matches COBOL &lt; ZERO. Negative inputs set Y. Other inputs preserve the existing flag. Equivalence also depends on a matching exact numeric input contract.</x:v>
+      </x:c>
+      <x:c r="E33" s="39" t="str">
+        <x:v>Implemented but unverified</x:v>
+      </x:c>
+      <x:c r="F33" s="39" t="str">
+        <x:v>Illustration only; nothing executed.
+Unit tests: unavailable.
+Observed mainframe parity: unavailable.
+Next: validate the numeric contract and 100 positive + 100 negative distinct cases. Owner: QA.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="27" customHeight="1">
+      <x:c r="A34" s="2"/>
+      <x:c r="B34" s="2"/>
+      <x:c r="C34" s="2"/>
+      <x:c r="D34" s="2"/>
+      <x:c r="E34" s="2"/>
+      <x:c r="F34" s="2"/>
+    </x:row>
+    <x:row r="35" ht="27" customHeight="1">
+      <x:c r="A35" s="2"/>
+      <x:c r="B35" s="2"/>
+      <x:c r="C35" s="2"/>
+      <x:c r="D35" s="2"/>
+      <x:c r="E35" s="2"/>
+      <x:c r="F35" s="2"/>
+    </x:row>
+    <x:row r="36" ht="27" customHeight="1">
+      <x:c r="A36" s="2"/>
+      <x:c r="B36" s="2"/>
+      <x:c r="C36" s="2"/>
+      <x:c r="D36" s="2"/>
+      <x:c r="E36" s="2"/>
+      <x:c r="F36" s="2"/>
+    </x:row>
+    <x:row r="37" ht="27" customHeight="1">
+      <x:c r="A37" s="2"/>
+      <x:c r="B37" s="2"/>
+      <x:c r="C37" s="2"/>
+      <x:c r="D37" s="2"/>
+      <x:c r="E37" s="2"/>
+      <x:c r="F37" s="2"/>
+    </x:row>
+    <x:row r="38" ht="27" customHeight="1">
+      <x:c r="A38" s="2"/>
+      <x:c r="B38" s="2"/>
+      <x:c r="C38" s="2"/>
+      <x:c r="D38" s="2"/>
+      <x:c r="E38" s="2"/>
+      <x:c r="F38" s="2"/>
+    </x:row>
+    <x:row r="39" ht="27" customHeight="1">
+      <x:c r="A39" s="2"/>
+      <x:c r="B39" s="2"/>
+      <x:c r="C39" s="2"/>
+      <x:c r="D39" s="2"/>
+      <x:c r="E39" s="2"/>
+      <x:c r="F39" s="2"/>
+    </x:row>
+  </x:sheetData>
+  <x:conditionalFormatting sqref="E7:E26">
+    <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Missing"/>
+    <x:cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Partial"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="E7:E26">
+      <x:formula1>"Missing,Partial,Implemented but unverified,Verified with evidence,Approved change/removal,Unknown,Non-executable source"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfca64362199a4dbf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add executable rule validation and reproducible evidence tools
Provide a whole-application operating guide and five small local utilities for compatibility receipts, every-rule data cases, captured-record replay, migration facts and instruction regression scoring. Align agent guidance and the review workbook with 100 positive and 100 negative cases for every executable rule.

Verified 105 local regressions and a 400-case synthetic example. Real Opus, application and mainframe acceptance remain separate workstation gates.
</commit_message>
<xml_diff>
--- a/examples/PTS_Modernization_Review_Template.xlsx
+++ b/examples/PTS_Modernization_Review_Template.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SME Review" sheetId="1" r:id="R7e3f523752e642c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Process Intake" sheetId="2" r:id="R21135b8b49e142d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Converted Inventory" sheetId="3" r:id="R65e343c42fdd42b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Evidence" sheetId="4" r:id="R9a30ba3c30cf481b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow" sheetId="5" r:id="Ref2c3834fbc14444"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Illustrative Review" sheetId="6" r:id="Rc7268194e2414807"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Catalog" sheetId="7" r:id="R67efac0c38894341"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Map" sheetId="8" r:id="Rc5677825de58492f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Analysis" sheetId="9" r:id="Rb1dd8110e95c4e76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Home" sheetId="10" r:id="R92c9e17623a44200"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Record Trace" sheetId="11" r:id="R04a335cbd2f541ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Manifest" sheetId="12" r:id="R841a54c5aa954282"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Record Index" sheetId="13" r:id="R2977280f5898460f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trace Events" sheetId="14" r:id="Rce6dc3e5ef8948e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SME Review" sheetId="1" r:id="Raf7f451aa42f43af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Process Intake" sheetId="2" r:id="R59c5d77bea78447b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Converted Inventory" sheetId="3" r:id="Re9e0f81858c3434f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule Evidence" sheetId="4" r:id="R92567733dc824d05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow" sheetId="5" r:id="R88599b8bcaea41a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Illustrative Review" sheetId="6" r:id="Rf1be1d3c81e34b6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Catalog" sheetId="7" r:id="R4fea73e7c53d4a25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agent Map" sheetId="8" r:id="Re4e01cdf88394b30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Analysis" sheetId="9" r:id="Re29c9495f3154199"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Home" sheetId="10" r:id="R330e398311bb46d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Record Trace" sheetId="11" r:id="Ra62df12932e54fa5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Manifest" sheetId="12" r:id="Rdf6f4e662e1047fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Record Index" sheetId="13" r:id="R23de288f9ec84a63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trace Events" sheetId="14" r:id="R2633d3d4488f40c6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -779,7 +779,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="7">
+  <x:dxfs count="9">
     <x:dxf>
       <x:font>
         <x:color rgb="FF9C2F2F"/>
@@ -821,6 +821,23 @@
       <x:fill>
         <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8E2929"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFBE5E3"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF1CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -919,11 +936,11 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="UnitDataCases" displayName="UnitDataCases" ref="A6:N26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="UnitDataCases" displayName="UnitDataCases" ref="A6:N26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A6:N26"/>
   <x:tableColumns count="14">
     <x:tableColumn id="1" name="Case ID"/>
-    <x:tableColumn id="2" name="Business rule / technical unit ID"/>
+    <x:tableColumn id="2" name="Executable rule ID"/>
     <x:tableColumn id="3" name="Program / test version"/>
     <x:tableColumn id="4" name="Case category"/>
     <x:tableColumn id="5" name="Original file / hash / lines"/>
@@ -1082,7 +1099,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ConvertedInventory" displayName="ConvertedInventory" ref="A6:Q26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="ConvertedInventory" displayName="ConvertedInventory" ref="A6:Q26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A6:Q26"/>
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="Program / component ID"/>
@@ -1090,7 +1107,7 @@
     <x:tableColumn id="3" name="Conversion status"/>
     <x:tableColumn id="4" name="Original source / hash / lines"/>
     <x:tableColumn id="5" name="Target modules / symbols"/>
-    <x:tableColumn id="6" name="Converted business rule IDs"/>
+    <x:tableColumn id="6" name="Converted executable rule IDs"/>
     <x:tableColumn id="7" name="Technical unit IDs"/>
     <x:tableColumn id="8" name="Databases / tables / migrations"/>
     <x:tableColumn id="9" name="Dependency fingerprint"/>
@@ -1108,10 +1125,10 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="RuleEvidence" displayName="RuleEvidence" ref="A6:T26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="RuleEvidence" displayName="RuleEvidence" ref="A6:T26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A6:T26"/>
   <x:tableColumns count="20">
-    <x:tableColumn id="1" name="Business rule ID"/>
+    <x:tableColumn id="1" name="Executable rule ID"/>
     <x:tableColumn id="2" name="Program ID / version"/>
     <x:tableColumn id="3" name="Source file / hash / lines"/>
     <x:tableColumn id="4" name="Positive and negative definitions"/>
@@ -2078,7 +2095,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52921cacfb154c97"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9205e8b2612c44cf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2242,12 +2259,12 @@
     <x:row r="18" ht="27" customHeight="1">
       <x:c r="A18" s="84"/>
       <x:c r="B18" s="46" t="str">
-        <x:f>IFERROR(HYPERLINK("#'Rule Evidence'!A1","Has each business rule passed its data cases?"),"Has each business rule passed its data cases?")</x:f>
-        <x:v>Has each business rule passed its data cases?</x:v>
+        <x:f>IFERROR(HYPERLINK("#'Rule Evidence'!A1","Has each executable rule passed its data cases?"),"Has each executable rule passed its data cases?")</x:f>
+        <x:v>Has each executable rule passed its data cases?</x:v>
       </x:c>
       <x:c r="C18" s="84"/>
       <x:c r="D18" s="89" t="str">
-        <x:v>Review 100 distinct positive and 100 negative passing cases per business rule. Technical operations use appropriate checks.</x:v>
+        <x:v>Every executable business, technical or mixed rule requires 100 distinct positive and 100 distinct negative passing cases.</x:v>
       </x:c>
       <x:c r="E18" s="89"/>
     </x:row>
@@ -26078,10 +26095,10 @@
     <x:mergeCell ref="A20:I20"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="C23:C1022">
-    <x:cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Error"/>
+    <x:cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="Error"/>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="A14:I14">
-    <x:cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="Partial"/>
+    <x:cfRule type="containsText" dxfId="8" priority="2" operator="containsText" text="Partial"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -27311,7 +27328,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22129718ed7a4e5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba0620dd95564c0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28806,7 +28823,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R446ab07532ad4bc6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R013c84a74a434e85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -30754,7 +30771,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69da49b5f79942b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1df97844ab654ed1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31518,8 +31535,8 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95330162686a48e0"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1e60c3470e8a43bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c4f4c40fb224e85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5907ce3216db428e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31674,7 +31691,7 @@
         <x:v>Target modules / symbols</x:v>
       </x:c>
       <x:c r="F6" s="66" t="str">
-        <x:v>Converted business rule IDs</x:v>
+        <x:v>Converted executable rule IDs</x:v>
       </x:c>
       <x:c r="G6" s="66" t="str">
         <x:v>Technical unit IDs</x:v>
@@ -32181,7 +32198,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0fe1743d4b5d413f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27a20538b65243bd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32245,7 +32262,7 @@
     </x:row>
     <x:row r="2" ht="32" customHeight="1">
       <x:c r="A2" s="47" t="str">
-        <x:v>Business rule unit test evidence</x:v>
+        <x:v>Executable rule unit test evidence</x:v>
       </x:c>
       <x:c r="B2" s="5"/>
       <x:c r="C2" s="5"/>
@@ -32269,7 +32286,7 @@
     </x:row>
     <x:row r="3" ht="27" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>Per business rule: 100 distinct positive + 100 distinct negative data cases derived from COBOL. Re-runs add no cases.</x:v>
+        <x:v>Every executable business, technical or mixed rule: 100 distinct positive + 100 distinct negative data cases from source. Re-runs add no cases.</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -32345,7 +32362,7 @@
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
       <x:c r="A6" s="65" t="str">
-        <x:v>Business rule ID</x:v>
+        <x:v>Executable rule ID</x:v>
       </x:c>
       <x:c r="B6" s="66" t="str">
         <x:v>Program ID / version</x:v>
@@ -33013,7 +33030,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raea37b59a93845e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71c55aa9e6b544ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33165,7 +33182,7 @@
         <x:v>QA + DevOps + analytics</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
-        <x:v>Create 100 positive and 100 negative distinct data cases per business rule from COBOL. Test technical contracts appropriately. Capture actual results and reconcile permitted legacy evidence. Existing remote denies remain effective.</x:v>
+        <x:v>Create 100 distinct positive and 100 distinct negative cases for every executable business, technical or mixed rule from source. Capture actual results and reconcile permitted legacy evidence. Existing remote denies remain effective.</x:v>
       </x:c>
       <x:c r="D12" s="17" t="str">
         <x:v>Case Catalog + Rule Evidence + run evidence</x:v>
@@ -33339,7 +33356,7 @@
         <x:v>Program owner</x:v>
       </x:c>
       <x:c r="C26" s="16" t="str">
-        <x:v>Business rule cases: 100 positive + 100 negative each. Separate technical, adapter, integration and performance tests.</x:v>
+        <x:v>Every executable business, technical or mixed rule: 100 positive + 100 negative cases. Also test adapters, integration and performance.</x:v>
       </x:c>
       <x:c r="D26" s="16" t="str">
         <x:v>Replayable fixtures, expected data and reference versions</x:v>
@@ -33465,13 +33482,13 @@
     </x:row>
     <x:row r="37" ht="104" customHeight="1">
       <x:c r="A37" s="16" t="str">
-        <x:v>Business rules validated</x:v>
+        <x:v>Executable rules validated</x:v>
       </x:c>
       <x:c r="B37" s="16" t="str">
         <x:v>Validation</x:v>
       </x:c>
       <x:c r="C37" s="16" t="str">
-        <x:v>For each business rule, create and pass 100 positive and 100 negative distinct data cases derived from COBOL. Negative cases assert the correct negative outcome; they are not failing tests. Repeated runs do not add cases.</x:v>
+        <x:v>Every executable business, technical or mixed rule must pass 100 distinct positive and 100 distinct negative source-derived cases. Negative cases assert the correct negative outcome. Repeated runs add no cases.</x:v>
       </x:c>
       <x:c r="D37" s="16" t="str">
         <x:v>Per-case inputs, expectations, actual results and source refs</x:v>
@@ -33704,7 +33721,7 @@
         <x:v>Account for every span. Technical behavior receives contract-based tests. Behavior-bearing declarations require target structure and verification. Inert text gets an explicit reason.</x:v>
       </x:c>
       <x:c r="D55" s="17" t="str">
-        <x:v>No 200-case quota for pure technical operations</x:v>
+        <x:v>Technical rules also require 100 positive + 100 negative cases</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="84" customHeight="1">
@@ -33880,11 +33897,11 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="5">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde0e8437f9ee48b7"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf366da943f6d4858"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc76580c80bf34bd6"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6648e389d84543f9"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R553aa83b24e1406c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raef42d7cbc3a4f56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b0c045bf1374244"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6efee16b6d84be9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c50b8018b6b4e12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab60397c1579440b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34278,7 +34295,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="N9" s="16" t="str">
-        <x:v>Technical test plan required; no 200-case quota</x:v>
+        <x:v>100 positive + 100 negative technical cases required</x:v>
       </x:c>
       <x:c r="O9" s="16" t="str">
         <x:v>Example processes P001 and P002</x:v>
@@ -34409,7 +34426,7 @@
     </x:row>
     <x:row r="13" ht="27" customHeight="1">
       <x:c r="A13" s="2" t="str">
-        <x:v>100 distinct positive and 100 distinct negative unit data cases are required per business rule. Repeated executions do not count.</x:v>
+        <x:v>Every executable business, technical or mixed rule requires 100 distinct positive and 100 distinct negative cases. Repeated runs add no cases.</x:v>
       </x:c>
       <x:c r="B13" s="2"/>
       <x:c r="C13" s="2"/>
@@ -34646,7 +34663,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R648731e3c8c542ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05c2e8934dfd4b55"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -34771,7 +34788,7 @@
         <x:v>Case ID</x:v>
       </x:c>
       <x:c r="B6" s="66" t="str">
-        <x:v>Business rule / technical unit ID</x:v>
+        <x:v>Executable rule ID</x:v>
       </x:c>
       <x:c r="C6" s="66" t="str">
         <x:v>Program / test version</x:v>
@@ -35281,7 +35298,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc53b90911c724252"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58105e8b19454bdb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35542,7 +35559,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38d270cbcda44f82"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb056b1d2a44d446a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -35968,7 +35985,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c091f5081c349f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47373cd8e5c147b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>